<commit_message>
mqtt improvements and code cleanup
</commit_message>
<xml_diff>
--- a/ws_mqtt_proto/app_proto.xlsx
+++ b/ws_mqtt_proto/app_proto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\esp32\esp32_common\ws_mqtt_proto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB584BA3-3C4B-4419-A56F-91F3969F0D8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8D5D265-3240-4C54-B98E-E3F4C3C0FF9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1965" windowWidth="25170" windowHeight="15345" xr2:uid="{F18B4279-3DD4-4A7B-B6C0-9AE4AF60F1CA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{F18B4279-3DD4-4A7B-B6C0-9AE4AF60F1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="82">
   <si>
     <t>ver</t>
   </si>
@@ -281,6 +281,15 @@
 sta_ssid
 sta_rssi
 time</t>
+  </si>
+  <si>
+    <t>CMD_QUERYSTATE</t>
+  </si>
+  <si>
+    <t>CMD_SETCONF</t>
+  </si>
+  <si>
+    <t>parameter name</t>
   </si>
 </sst>
 </file>
@@ -711,7 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39BBDBE0-EF55-4425-BC9A-1895DB5EC3FA}">
-  <dimension ref="B2:Q25"/>
+  <dimension ref="B2:Q32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.5703125" bestFit="1" customWidth="1"/>
@@ -1108,7 +1117,12 @@
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="G15" s="1"/>
+      <c r="F15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>81</v>
+      </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="P15" t="s">
@@ -1119,6 +1133,16 @@
       </c>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
       <c r="P16" t="s">
         <v>65</v>
       </c>
@@ -1126,199 +1150,87 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B18" s="2">
-        <v>1</v>
-      </c>
-      <c r="C18" s="2">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P24">
+        <f>7500/230</f>
+        <v>32.608695652173914</v>
+      </c>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B25" s="2">
+        <v>1</v>
+      </c>
+      <c r="C25" s="2">
         <v>9</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D25" s="2">
         <v>0</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="2" t="s">
+      <c r="E25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="H25" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B19" s="1">
-        <v>1</v>
-      </c>
-      <c r="C19" s="1">
-        <v>8</v>
-      </c>
-      <c r="D19" s="1">
-        <v>0</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B20" s="10">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10">
-        <v>9</v>
-      </c>
-      <c r="D20" s="10">
-        <v>0</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I20" t="s">
-        <v>17</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="J22" s="1"/>
-    </row>
-    <row r="23" spans="2:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="B23" s="2">
-        <v>1</v>
-      </c>
-      <c r="C23" s="2">
-        <v>7</v>
-      </c>
-      <c r="D23" s="2">
-        <v>0</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B24" s="1">
-        <v>1</v>
-      </c>
-      <c r="C24" s="1">
-        <v>9</v>
-      </c>
-      <c r="D24" s="1">
-        <v>0</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="1">
-        <v>1</v>
-      </c>
-      <c r="C25" s="1">
-        <v>9</v>
-      </c>
-      <c r="D25" s="1">
-        <v>0</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>15</v>
@@ -1326,15 +1238,199 @@
       <c r="J25" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="P25">
+        <f>9*3.14*2.5</f>
+        <v>70.650000000000006</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B26" s="1">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1">
+        <v>8</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P26">
+        <f>P25*230</f>
+        <v>16249.500000000002</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B27" s="10">
+        <v>1</v>
+      </c>
+      <c r="C27" s="10">
+        <v>9</v>
+      </c>
+      <c r="D27" s="10">
+        <v>0</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="P28">
+        <f>70*70*0.05</f>
+        <v>245</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="J29" s="1"/>
+    </row>
+    <row r="30" spans="2:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="B30" s="2">
+        <v>1</v>
+      </c>
+      <c r="C30" s="2">
+        <v>7</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B31" s="1">
+        <v>1</v>
+      </c>
+      <c r="C31" s="1">
+        <v>9</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B32" s="1">
+        <v>1</v>
+      </c>
+      <c r="C32" s="1">
+        <v>9</v>
+      </c>
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="F20:F22"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D27:D29"/>
+    <mergeCell ref="E27:E29"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="F27:F29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="C27:C29"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>